<commit_message>
feat: migrate to v5 agent contracts and demo loop
</commit_message>
<xml_diff>
--- a/reports/evaluation/latest-baseline.xlsx
+++ b/reports/evaluation/latest-baseline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="agent_latency" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="agent_latency" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,13 +446,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>200</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -462,13 +462,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C3" t="n">
         <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -478,13 +478,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3875</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="8">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5701</v>
+        <v>1920</v>
       </c>
     </row>
   </sheetData>
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,6 +570,45 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>content_generation_agent</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>572</v>
+      </c>
+      <c r="C2" t="n">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>knowledge_retrieval_agent</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>146</v>
+      </c>
+      <c r="C3" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>review_validation_agent</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>482</v>
+      </c>
+      <c r="C4" t="n">
+        <v>526</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>